<commit_message>
new commit with msi
</commit_message>
<xml_diff>
--- a/templates/New Worksheet.xlsx
+++ b/templates/New Worksheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pamodana Wijewantha\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\TeaCollectionApp\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{912DFCAE-F551-401D-9BE9-E264B7D06E65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94680235-D2EB-438F-8AE2-E7746191B509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4875" windowWidth="29040" windowHeight="15720" xr2:uid="{A0F26370-F9FD-4153-8EAB-E4772B52117B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A0F26370-F9FD-4153-8EAB-E4772B52117B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,23 +29,17 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="217">
   <si>
     <t>Customer Code</t>
   </si>
   <si>
     <t>Customer Name</t>
-  </si>
-  <si>
-    <t>29(Poya)</t>
   </si>
   <si>
     <t xml:space="preserve">TA001 </t>
@@ -787,9 +781,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -827,7 +821,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -933,7 +927,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1075,7 +1069,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1181,8 +1175,8 @@
       <c r="AD1" s="2">
         <v>28</v>
       </c>
-      <c r="AE1" s="2" t="s">
-        <v>2</v>
+      <c r="AE1" s="2">
+        <v>29</v>
       </c>
       <c r="AF1" s="2">
         <v>30</v>
@@ -1193,7 +1187,7 @@
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
@@ -1230,7 +1224,7 @@
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
@@ -1267,10 +1261,10 @@
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>6</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -1306,10 +1300,10 @@
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>8</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -1345,7 +1339,7 @@
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1"/>
@@ -1382,10 +1376,10 @@
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>11</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -1421,10 +1415,10 @@
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -1460,10 +1454,10 @@
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -1499,10 +1493,10 @@
     </row>
     <row r="10" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -1538,10 +1532,10 @@
     </row>
     <row r="11" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -1577,10 +1571,10 @@
     </row>
     <row r="12" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
@@ -1616,10 +1610,10 @@
     </row>
     <row r="13" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="1" t="s">
         <v>22</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>23</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -1655,10 +1649,10 @@
     </row>
     <row r="14" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>24</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>25</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
@@ -1694,10 +1688,10 @@
     </row>
     <row r="15" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>27</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
@@ -1733,10 +1727,10 @@
     </row>
     <row r="16" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
@@ -1772,10 +1766,10 @@
     </row>
     <row r="17" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
@@ -1811,10 +1805,10 @@
     </row>
     <row r="18" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>33</v>
       </c>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
@@ -1850,10 +1844,10 @@
     </row>
     <row r="19" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>34</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>35</v>
       </c>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
@@ -1889,10 +1883,10 @@
     </row>
     <row r="20" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>37</v>
       </c>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
@@ -1928,10 +1922,10 @@
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
@@ -1967,10 +1961,10 @@
     </row>
     <row r="22" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -2006,10 +2000,10 @@
     </row>
     <row r="23" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>42</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -2045,10 +2039,10 @@
     </row>
     <row r="24" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -2084,10 +2078,10 @@
     </row>
     <row r="25" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -2123,10 +2117,10 @@
     </row>
     <row r="26" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -2162,10 +2156,10 @@
     </row>
     <row r="27" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>50</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -2201,10 +2195,10 @@
     </row>
     <row r="28" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
@@ -2240,10 +2234,10 @@
     </row>
     <row r="29" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>55</v>
       </c>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
@@ -2279,10 +2273,10 @@
     </row>
     <row r="30" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>57</v>
       </c>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
@@ -2318,10 +2312,10 @@
     </row>
     <row r="31" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>58</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>59</v>
       </c>
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
@@ -2357,10 +2351,10 @@
     </row>
     <row r="32" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>61</v>
       </c>
       <c r="C32" s="1"/>
       <c r="D32" s="1"/>
@@ -2396,10 +2390,10 @@
     </row>
     <row r="33" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="C33" s="1"/>
       <c r="D33" s="1"/>
@@ -2435,10 +2429,10 @@
     </row>
     <row r="34" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>64</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="C34" s="1"/>
       <c r="D34" s="1"/>
@@ -2474,10 +2468,10 @@
     </row>
     <row r="35" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>66</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="C35" s="1"/>
       <c r="D35" s="1"/>
@@ -2513,10 +2507,10 @@
     </row>
     <row r="36" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>69</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
@@ -2552,10 +2546,10 @@
     </row>
     <row r="37" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37" s="1" t="s">
         <v>70</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>71</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
@@ -2591,10 +2585,10 @@
     </row>
     <row r="38" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
@@ -2630,10 +2624,10 @@
     </row>
     <row r="39" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" s="1" t="s">
         <v>74</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>75</v>
       </c>
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
@@ -2669,10 +2663,10 @@
     </row>
     <row r="40" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B40" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
@@ -2708,10 +2702,10 @@
     </row>
     <row r="41" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B41" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
@@ -2747,10 +2741,10 @@
     </row>
     <row r="42" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>81</v>
       </c>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -2786,10 +2780,10 @@
     </row>
     <row r="43" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>83</v>
       </c>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
@@ -2825,10 +2819,10 @@
     </row>
     <row r="44" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>85</v>
       </c>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
@@ -2864,10 +2858,10 @@
     </row>
     <row r="45" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B45" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
@@ -2903,10 +2897,10 @@
     </row>
     <row r="46" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B46" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="B46" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
@@ -2942,10 +2936,10 @@
     </row>
     <row r="47" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B47" s="1" t="s">
         <v>90</v>
-      </c>
-      <c r="B47" s="1" t="s">
-        <v>91</v>
       </c>
       <c r="C47" s="1"/>
       <c r="D47" s="1"/>
@@ -2981,10 +2975,10 @@
     </row>
     <row r="48" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B48" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>93</v>
       </c>
       <c r="C48" s="1"/>
       <c r="D48" s="1"/>
@@ -3020,10 +3014,10 @@
     </row>
     <row r="49" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B49" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>95</v>
       </c>
       <c r="C49" s="1"/>
       <c r="D49" s="1"/>
@@ -3059,10 +3053,10 @@
     </row>
     <row r="50" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>96</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>97</v>
       </c>
       <c r="C50" s="1"/>
       <c r="D50" s="1"/>
@@ -3098,10 +3092,10 @@
     </row>
     <row r="51" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B51" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>99</v>
       </c>
       <c r="C51" s="1"/>
       <c r="D51" s="1"/>
@@ -3137,10 +3131,10 @@
     </row>
     <row r="52" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>101</v>
       </c>
       <c r="C52" s="1"/>
       <c r="D52" s="1"/>
@@ -3176,10 +3170,10 @@
     </row>
     <row r="53" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>102</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>103</v>
       </c>
       <c r="C53" s="1"/>
       <c r="D53" s="1"/>
@@ -3215,10 +3209,10 @@
     </row>
     <row r="54" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C54" s="1"/>
       <c r="D54" s="1"/>
@@ -3254,10 +3248,10 @@
     </row>
     <row r="55" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B55" s="1" t="s">
         <v>106</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>107</v>
       </c>
       <c r="C55" s="1"/>
       <c r="D55" s="1"/>
@@ -3293,10 +3287,10 @@
     </row>
     <row r="56" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B56" s="1" t="s">
         <v>108</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>109</v>
       </c>
       <c r="C56" s="1"/>
       <c r="D56" s="1"/>
@@ -3332,10 +3326,10 @@
     </row>
     <row r="57" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B57" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
@@ -3371,10 +3365,10 @@
     </row>
     <row r="58" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B58" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
@@ -3410,10 +3404,10 @@
     </row>
     <row r="59" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B59" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>115</v>
       </c>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
@@ -3449,10 +3443,10 @@
     </row>
     <row r="60" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B60" s="1" t="s">
         <v>116</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>117</v>
       </c>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
@@ -3488,10 +3482,10 @@
     </row>
     <row r="61" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B61" s="1" t="s">
         <v>118</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>119</v>
       </c>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
@@ -3527,10 +3521,10 @@
     </row>
     <row r="62" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>120</v>
-      </c>
-      <c r="B62" s="1" t="s">
-        <v>121</v>
       </c>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
@@ -3566,10 +3560,10 @@
     </row>
     <row r="63" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>122</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>123</v>
       </c>
       <c r="C63" s="1"/>
       <c r="D63" s="1"/>
@@ -3605,10 +3599,10 @@
     </row>
     <row r="64" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>124</v>
-      </c>
-      <c r="B64" s="1" t="s">
-        <v>125</v>
       </c>
       <c r="C64" s="1"/>
       <c r="D64" s="1"/>
@@ -3644,10 +3638,10 @@
     </row>
     <row r="65" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>126</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>127</v>
       </c>
       <c r="C65" s="1"/>
       <c r="D65" s="1"/>
@@ -3683,10 +3677,10 @@
     </row>
     <row r="66" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>128</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>129</v>
       </c>
       <c r="C66" s="1"/>
       <c r="D66" s="1"/>
@@ -3722,10 +3716,10 @@
     </row>
     <row r="67" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="C67" s="1"/>
       <c r="D67" s="1"/>
@@ -3761,7 +3755,7 @@
     </row>
     <row r="68" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B68" s="1"/>
       <c r="C68" s="1"/>
@@ -3798,10 +3792,10 @@
     </row>
     <row r="69" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>134</v>
       </c>
       <c r="C69" s="1"/>
       <c r="D69" s="1"/>
@@ -3837,10 +3831,10 @@
     </row>
     <row r="70" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>136</v>
       </c>
       <c r="C70" s="1"/>
       <c r="D70" s="1"/>
@@ -3876,10 +3870,10 @@
     </row>
     <row r="71" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B71" s="1" t="s">
         <v>137</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>138</v>
       </c>
       <c r="C71" s="1"/>
       <c r="D71" s="1"/>
@@ -3915,10 +3909,10 @@
     </row>
     <row r="72" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B72" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="C72" s="1"/>
       <c r="D72" s="1"/>
@@ -3954,10 +3948,10 @@
     </row>
     <row r="73" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B73" s="1" t="s">
         <v>141</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>142</v>
       </c>
       <c r="C73" s="1"/>
       <c r="D73" s="1"/>
@@ -3993,10 +3987,10 @@
     </row>
     <row r="74" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B74" s="1" t="s">
         <v>143</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>144</v>
       </c>
       <c r="C74" s="1"/>
       <c r="D74" s="1"/>
@@ -4032,10 +4026,10 @@
     </row>
     <row r="75" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>145</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>146</v>
       </c>
       <c r="C75" s="1"/>
       <c r="D75" s="1"/>
@@ -4071,10 +4065,10 @@
     </row>
     <row r="76" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B76" s="1" t="s">
         <v>147</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>148</v>
       </c>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
@@ -4110,10 +4104,10 @@
     </row>
     <row r="77" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B77" s="1" t="s">
         <v>149</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
@@ -4149,10 +4143,10 @@
     </row>
     <row r="78" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B78" s="1" t="s">
         <v>151</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>152</v>
       </c>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
@@ -4188,10 +4182,10 @@
     </row>
     <row r="79" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B79" s="1" t="s">
         <v>153</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>154</v>
       </c>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
@@ -4227,10 +4221,10 @@
     </row>
     <row r="80" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B80" s="1" t="s">
         <v>155</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>156</v>
       </c>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
@@ -4266,10 +4260,10 @@
     </row>
     <row r="81" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B81" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>158</v>
       </c>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
@@ -4305,10 +4299,10 @@
     </row>
     <row r="82" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B82" s="1" t="s">
         <v>159</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>160</v>
       </c>
       <c r="C82" s="1"/>
       <c r="D82" s="1"/>
@@ -4344,10 +4338,10 @@
     </row>
     <row r="83" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B83" s="1" t="s">
         <v>161</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>162</v>
       </c>
       <c r="C83" s="1"/>
       <c r="D83" s="1"/>
@@ -4383,10 +4377,10 @@
     </row>
     <row r="84" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="B84" s="1" t="s">
         <v>163</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>164</v>
       </c>
       <c r="C84" s="1"/>
       <c r="D84" s="1"/>
@@ -4422,10 +4416,10 @@
     </row>
     <row r="85" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B85" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="C85" s="1"/>
       <c r="D85" s="1"/>
@@ -4461,10 +4455,10 @@
     </row>
     <row r="86" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>168</v>
       </c>
       <c r="C86" s="1"/>
       <c r="D86" s="1"/>
@@ -4500,10 +4494,10 @@
     </row>
     <row r="87" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B87" s="1" t="s">
         <v>169</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>170</v>
       </c>
       <c r="C87" s="1"/>
       <c r="D87" s="1"/>
@@ -4539,10 +4533,10 @@
     </row>
     <row r="88" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B88" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>172</v>
       </c>
       <c r="C88" s="1"/>
       <c r="D88" s="1"/>
@@ -4578,10 +4572,10 @@
     </row>
     <row r="89" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B89" s="1" t="s">
         <v>173</v>
-      </c>
-      <c r="B89" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="C89" s="1"/>
       <c r="D89" s="1"/>
@@ -4617,10 +4611,10 @@
     </row>
     <row r="90" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B90" s="1" t="s">
         <v>175</v>
-      </c>
-      <c r="B90" s="1" t="s">
-        <v>176</v>
       </c>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
@@ -4656,10 +4650,10 @@
     </row>
     <row r="91" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B91" s="1" t="s">
         <v>177</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>178</v>
       </c>
       <c r="C91" s="1"/>
       <c r="D91" s="1"/>
@@ -4695,10 +4689,10 @@
     </row>
     <row r="92" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>179</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>180</v>
       </c>
       <c r="C92" s="1"/>
       <c r="D92" s="1"/>
@@ -4734,10 +4728,10 @@
     </row>
     <row r="93" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B93" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>182</v>
       </c>
       <c r="C93" s="1"/>
       <c r="D93" s="1"/>
@@ -4773,10 +4767,10 @@
     </row>
     <row r="94" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="B94" s="1" t="s">
         <v>183</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>184</v>
       </c>
       <c r="C94" s="1"/>
       <c r="D94" s="1"/>
@@ -4812,10 +4806,10 @@
     </row>
     <row r="95" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B95" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>186</v>
       </c>
       <c r="C95" s="1"/>
       <c r="D95" s="1"/>
@@ -4851,10 +4845,10 @@
     </row>
     <row r="96" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B96" s="1" t="s">
         <v>187</v>
-      </c>
-      <c r="B96" s="1" t="s">
-        <v>188</v>
       </c>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
@@ -4890,10 +4884,10 @@
     </row>
     <row r="97" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B97" s="1" t="s">
         <v>189</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>190</v>
       </c>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
@@ -4929,7 +4923,7 @@
     </row>
     <row r="98" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
@@ -4966,10 +4960,10 @@
     </row>
     <row r="99" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="B99" s="1" t="s">
         <v>192</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>193</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
@@ -5005,10 +4999,10 @@
     </row>
     <row r="100" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B100" s="1" t="s">
         <v>194</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>195</v>
       </c>
       <c r="C100" s="1"/>
       <c r="D100" s="1"/>
@@ -5044,10 +5038,10 @@
     </row>
     <row r="101" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="B101" s="1" t="s">
         <v>196</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>197</v>
       </c>
       <c r="C101" s="1"/>
       <c r="D101" s="1"/>
@@ -5083,10 +5077,10 @@
     </row>
     <row r="102" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B102" s="1" t="s">
         <v>198</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>199</v>
       </c>
       <c r="C102" s="1"/>
       <c r="D102" s="1"/>
@@ -5122,10 +5116,10 @@
     </row>
     <row r="103" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="B103" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="B103" s="1" t="s">
-        <v>201</v>
       </c>
       <c r="C103" s="1"/>
       <c r="D103" s="1"/>
@@ -5161,10 +5155,10 @@
     </row>
     <row r="104" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B104" s="1" t="s">
         <v>202</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>203</v>
       </c>
       <c r="C104" s="1"/>
       <c r="D104" s="1"/>
@@ -5200,10 +5194,10 @@
     </row>
     <row r="105" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="B105" s="1" t="s">
         <v>204</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>205</v>
       </c>
       <c r="C105" s="1"/>
       <c r="D105" s="1"/>
@@ -5239,10 +5233,10 @@
     </row>
     <row r="106" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B106" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="B106" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="C106" s="1"/>
       <c r="D106" s="1"/>
@@ -5278,10 +5272,10 @@
     </row>
     <row r="107" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="B107" s="1" t="s">
         <v>208</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>209</v>
       </c>
       <c r="C107" s="1"/>
       <c r="D107" s="1"/>
@@ -5317,10 +5311,10 @@
     </row>
     <row r="108" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B108" s="1" t="s">
         <v>210</v>
-      </c>
-      <c r="B108" s="1" t="s">
-        <v>211</v>
       </c>
       <c r="C108" s="1"/>
       <c r="D108" s="1"/>
@@ -5356,10 +5350,10 @@
     </row>
     <row r="109" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="B109" s="1" t="s">
         <v>212</v>
-      </c>
-      <c r="B109" s="1" t="s">
-        <v>213</v>
       </c>
       <c r="C109" s="1"/>
       <c r="D109" s="1"/>
@@ -5395,10 +5389,10 @@
     </row>
     <row r="110" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B110" s="1" t="s">
         <v>214</v>
-      </c>
-      <c r="B110" s="1" t="s">
-        <v>215</v>
       </c>
       <c r="C110" s="1"/>
       <c r="D110" s="1"/>
@@ -5434,10 +5428,10 @@
     </row>
     <row r="111" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B111" s="1" t="s">
         <v>216</v>
-      </c>
-      <c r="B111" s="1" t="s">
-        <v>217</v>
       </c>
       <c r="C111" s="1"/>
       <c r="D111" s="1"/>

</xml_diff>